<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-08 La brioche de Raphaël
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-08.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-08.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La brioche sous la lampe de Raphaël</t>
+          <t>La brioche de Raphaël</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>rue mouillée, boulangerie le soir</t>
+          <t>rue mouillée, réverbère, pavés, boulangerie, odeur de beurre</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut la brioche floue dans la vitre embuée. Il dit bonjour, s'il te plaît, merci. Le sac reste tiède.</t>
+          <t>Une flaque ronde tient un cercle jaune. Sur le verre, un éclat de réverbère brille. Raphaël veut la brioche floue maintenant. Il avance trop vite, sans le mot : la boulangère ne tourne pas. Il refuse de foncer, dit bonjour. Merci vécu. Dehors, le vent gonfle le sachet comme des ailes. Il refuse, serre. Sur le verre, l'éclat de réverbère tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une gouttière chante dans la rue. L'eau tombe dans un seau, une goutte après l'autre. Une odeur de sucre sort sous la porte. Papa tient un parapluie encore mouillé. Une goutte glisse le long du tissu. Tu entends la gouttière, Raphaël ? Elle chante, maman. Dans le seau. La boulangerie a une lampe ronde. La vitre est embuée, tout en bas. Une brioche dorée s'y dessine, un peu floue. Je la vois, papa. Oui. On entre. En ce moment, ils poussent la porte. Une cloche fait ding, tout doux. L'air est chaud, comme une couverture. Ça sent la brioche et le sucre. La boulangère range des pains ronds. Elle a les mains pleines. On attend un peu. Raphaël s'arrête sous la lampe. Un sac en papier attend sur le marbre. Il est vide, ce sac. Pour la brioche, après. La boulangère pose un pain. Elle se tourne, le torchon à la main. Tu demandes, Raphaël.</t>
+          <t>Une flaque ronde tient un cercle jaune. La rue est mouillée, un peu sombre. Les pavés luisent sous les pas. Ils brillent, papa. Tu les vois, sous tes pieds ? Une odeur de beurre court sur le trottoir. Ça sent le beurre, maman. Oui, tout le long de la rue. Un sac en papier danse près d'une grille. Maman rattrape le sac du bout des doigts. Il voulait s'envoler. Il a des ailes, maman. Des ailes de papier, oui. Le ciel est bas, un peu gris. Le réverbère jaune trempe l'eau de la rue. Sur le verre, un éclat de réverbère brille. Il est blanc, papa. C'est la lampe, dans l'eau. Tu le touches, Raphaël ? Raphaël pose un doigt sur le verre. Le verre est froid, un peu mouillé. Il pique un peu. On avance. La boulangerie a une lampe ronde, au-dessus de la porte. La vitre est embuée, tout en bas. Une brioche dorée s'y dessine, un peu floue. Je la vois, maman. Elle est derrière le verre. Je la veux, maintenant ! On pousse la porte ? Oui, maintenant ! En ce moment, Raphaël pose la main sur la porte. La cloche fait ding, un peu fort. L'air chaud touche les joues. Ça sent la brioche et le beurre. La boulangère range des pains ronds. Celle-là, maintenant ! Raphaël avance trop vite vers le comptoir. Sa voix se mélange à la cloche. Oh. La boulangère ne tourne pas la tête. Le torchon reste dans ses mains. La brioche reste floue, derrière le verre. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elle ne m'entend pas, papa. Tu la vois, Raphaël ? Papa se baisse à sa hauteur. L'éclat de réverbère tremble, puis tient. Les épaules de Raphaël tombent un peu. Le sac de dehors danse, là. Le mien sera chaud.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une gouttière chante dans la rue. L'eau tombe dans un seau, une goutte après l'autre. Une odeur de sucre sort sous la porte. Papa tient un parapluie encore mouillé. Une goutte glisse le long du tissu. Tu entends la gouttière, Raphaël ? Elle chante, maman. Dans le seau. La boulangerie a une lampe ronde. La vitre est embuée, tout en bas. Une brioche dorée s'y dessine, un peu floue. Je la vois, papa. Oui. On entre. En ce moment, ils poussent la porte. Une cloche fait ding, tout doux. L'air est chaud, comme une couverture. Ça sent la brioche et le sucre. La boulangère range des pains ronds. Elle a les mains pleines. On attend un peu. Raphaël s'arrête sous la lampe. Un sac en papier attend sur le marbre. Il est vide, ce sac. Pour la brioche, après. La boulangère pose un pain. Elle se tourne, le torchon à la main. Tu demandes, Raphaël.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une flaque ronde tient un cercle jaune. La rue est mouillée, un peu sombre. Les pavés luisent sous les pas. Ils brillent, papa. Tu les vois, sous tes pieds ? Une odeur de beurre court sur le trottoir. Ça sent le beurre, maman. Oui, tout le long de la rue. Un sac en papier danse près d'une grille. Maman rattrape le sac du bout des doigts. Il voulait s'envoler. Il a des ailes, maman. Des ailes de papier, oui. Le ciel est bas, un peu gris. Le réverbère jaune trempe l'eau de la rue. Sur le verre, un &lt;emphasis level="moderate"&gt;éclat de réverbère&lt;/emphasis&gt; brille. Il est blanc, papa. C'est la lampe, dans l'eau. Tu le touches, Raphaël ? Raphaël pose un doigt sur le verre. Le verre est froid, un peu mouillé. Il pique un peu. On avance. La boulangerie a une lampe ronde, au-dessus de la porte. La vitre est embuée, tout en bas. Une brioche dorée s'y dessine, un peu floue. Je la vois, maman. Elle est derrière le verre. Je la veux, maintenant ! On pousse la porte ? Oui, maintenant ! En ce moment, Raphaël pose la main sur la porte. La cloche fait ding, un peu fort. L'air chaud touche les joues. Ça sent la brioche et le beurre. La boulangère range des pains ronds. Celle-là, maintenant ! Raphaël avance trop vite vers le comptoir. Sa voix se mélange à la cloche. Oh. La boulangère ne tourne pas la tête. Le torchon reste dans ses mains. La brioche reste floue, derrière le verre. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elle ne m'entend pas, papa. Tu la vois, Raphaël ? Papa se baisse à sa hauteur. L'éclat de réverbère tremble, puis tient. Les épaules de Raphaël tombent un peu. Le sac de dehors danse, là. Le mien sera chaud.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Pascal entre à la boulangerie avec maman. Ça sent le pain. Pascal dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Il dit s'il te plaît pour une brioche. Il dit merci. Maman sourit. La boulangère sourit. Pascal répète : bonjour, s'il te plaît, merci. Ils sortent. Pascal tient le sac. [pause]</t>
+          <t>Une flaque ronde tient un cercle jaune. La rue est mouillée, un peu sombre. Les pavés luisent sous les pas. Ils brillent, papa. Tu les vois, sous tes pieds ? Une odeur de beurre court sur le trottoir. Ça sent le beurre, maman. Oui, tout le long de la rue. Un sac en papier danse près d'une grille. Maman rattrape le sac du bout des doigts. Il voulait s'envoler. Il a des ailes, maman. Des ailes de papier, oui. Le ciel est bas, un peu gris. Le réverbère jaune trempe l'eau de la rue. Sur le verre, un &lt;emphasis&gt;éclat de réverbère&lt;/emphasis&gt; brille. Il est blanc, papa. C'est la lampe, dans l'eau. Tu le touches, Raphaël ? Raphaël pose un doigt sur le verre. Le verre est froid, un peu mouillé. Il pique un peu. On avance. La boulangerie a une lampe ronde, au-dessus de la porte. La vitre est embuée, tout en bas. Une brioche dorée s'y dessine, un peu floue. Je la vois, maman. Elle est derrière le verre. Je la veux, maintenant ! On pousse la porte ? Oui, maintenant ! En ce moment, Raphaël pose la main sur la porte. La cloche fait ding, un peu fort. L'air chaud touche les joues. Ça sent la brioche et le beurre. La boulangère range des pains ronds. Celle-là, maintenant ! Raphaël avance trop vite vers le comptoir. Sa voix se mélange à la cloche. Oh. La boulangère ne tourne pas la tête. Le torchon reste dans ses mains. La brioche reste floue, derrière le verre. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elle ne m'entend pas, papa. Tu la vois, Raphaël ? Papa se baisse à sa hauteur. L'éclat de réverbère tremble, puis tient. Les épaules de Raphaël tombent un peu. Le sac de dehors danse, là. Le mien sera chaud. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de réverbère</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,42 +1326,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_brioche_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une gouttière chante dans la rue.
-narrateur|L'eau tombe dans un seau, une goutte après l'autre.
-narrateur|Une odeur de sucre sort sous la porte.
-narrateur|Papa tient un parapluie encore mouillé.
-narrateur|Une goutte glisse le long du tissu.
-maman|Tu entends la gouttière, Raphaël ?
-enfant-m|Elle chante, maman.
-papa|Dans le seau.
-narrateur|La boulangerie a une lampe ronde.
+          <t>narrateur|Une flaque ronde tient un cercle jaune.
+narrateur|La rue est mouillée, un peu sombre.
+narrateur|Les pavés luisent sous les pas.
+enfant-m|Ils brillent, papa.
+papa|Tu les vois, sous tes pieds ?
+narrateur|Une odeur de beurre court sur le trottoir.
+enfant-m|Ça sent le beurre, maman.
+maman|Oui, tout le long de la rue.
+narrateur|Un sac en papier danse près d'une grille.
+narrateur|Maman rattrape le sac du bout des doigts.
+maman|Il voulait s'envoler.
+enfant-m|Il a des ailes, maman.
+papa|Des ailes de papier, oui.
+narrateur|Le ciel est bas, un peu gris.
+narrateur|Le réverbère jaune trempe l'eau de la rue.
+narrateur|Sur le verre, un éclat de réverbère brille.
+enfant-m|Il est blanc, papa.
+papa|C'est la lampe, dans l'eau.
+maman|Tu le touches, Raphaël ?
+narrateur|Raphaël pose un doigt sur le verre.
+narrateur|Le verre est froid, un peu mouillé.
+enfant-m|Il pique un peu.
+papa|On avance.
+narrateur|La boulangerie a une lampe ronde, au-dessus de la porte.
 narrateur|La vitre est embuée, tout en bas.
 narrateur|Une brioche dorée s'y dessine, un peu floue.
-enfant-m|Je la vois, papa.
-maman|Oui.
-papa|On entre.
-narrateur|En ce moment, ils poussent la porte.
-narrateur|Une cloche fait ding, tout doux.
-narrateur|L'air est chaud, comme une couverture.
-narrateur|Ça sent la brioche et le sucre.
+enfant-m|Je la vois, maman.
+maman|Elle est derrière le verre.
+enfant-m|Je la veux, maintenant !
+papa|On pousse la porte ?
+enfant-m|Oui, maintenant !
+narrateur|En ce moment, Raphaël pose la main sur la porte.
+narrateur|La cloche fait ding, un peu fort.
+narrateur|L'air chaud touche les joues.
+narrateur|Ça sent la brioche et le beurre.
 narrateur|La boulangère range des pains ronds.
-maman|Elle a les mains pleines.
-papa|On attend un peu.
-narrateur|Raphaël s'arrête sous la lampe.
-narrateur|Un sac en papier attend sur le marbre.
-enfant-m|Il est vide, ce sac.
-papa|Pour la brioche, après.
-narrateur|La boulangère pose un pain.
-narrateur|Elle se tourne, le torchon à la main.
-maman|Tu demandes, Raphaël.</t>
+enfant-m|Celle-là, maintenant !
+narrateur|Raphaël avance trop vite vers le comptoir.
+narrateur|Sa voix se mélange à la cloche.
+enfant-m|Oh.
+narrateur|La boulangère ne tourne pas la tête.
+narrateur|Le torchon reste dans ses mains.
+narrateur|La brioche reste floue, derrière le verre.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Elle ne m'entend pas, papa.
+papa|Tu la vois, Raphaël ?
+narrateur|Papa se baisse à sa hauteur.
+narrateur|L'éclat de réverbère tremble, puis tient.
+narrateur|Les épaules de Raphaël tombent un peu.
+maman|Le sac de dehors danse, là.
+enfant-m|Le mien sera chaud.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>gouttiere,cloche</t>
+          <t>pas,cloche</t>
         </is>
       </c>
     </row>
@@ -1388,17 +1416,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut la brioche. Que dit-il ?</t>
+          <t>Raphaël salue. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut la brioche. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël &lt;emphasis level="moderate"&gt;salue&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Pascal salue. Quels mots dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël &lt;emphasis&gt;salue&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1423,7 +1451,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit bonjour. Que dit Raphaël ?</t>
+          <t>Il dit bonjour. Quels mots dit Raphaël ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1461,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1472,7 +1500,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1487,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>salue</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1529,23 +1561,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_dit_bonjour; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël veut la brioche.
-narrateur|Que dit-il ?</t>
+          <t>narrateur|Raphaël salue.
+narrateur|Quels mots dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1572,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une brioche, s'il te plaît. Celle de la vitre. La boulangère glisse la brioche dans un sac. Le papier craque, un peu gras. Merci. Merci. Raphaël tient le sac à deux mains. Le fond du sac est tiède. Elle est chaude, maman. Oui. Un grain de sucre sur ton pouce. Il brille. Tu le goûtes ? Il est sucré. Ils restent un moment près de la vitre. Raphaël dessine un petit rond du doigt. La brioche n'est plus floue, dehors. Elle est dans le sac, maintenant. On garde le sac au chaud. Oui, maman.</t>
+          <t>Raphaël avance trop vite vers le comptoir. La brioche, maintenant ! Sa voix se mélange à la cloche. Oh. Le torchon ne bouge pas. Le sourire ne revient pas. Raphaël refuse de foncer. Il recule d'un pas, près du bois. Tu veux venir près du bois ? Papa reste à sa hauteur. Raphaël écoute la cloche, un instant. Par la vitre, l'éclat de réverbère brille. Bonjour. Bonjour. Une brioche, s'il te plaît. Celle de la vitre. Derrière le bois, une main se tend. Le papier enveloppe la brioche. Le sachet est chaud contre le manteau. Merci. Merci, Raphaël. Papa a entendu toute la phrase. Le ventre de Raphaël se desserre. Elle est chaude, maman. Tu as les mains dessus ? Oui, maman. Le papier est un peu gras, un peu tiède. Ça sent le beurre. On sort ? Oui, maman. Raphaël tient le sachet à deux mains. Le fond du sac est tiède.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une brioche, s'il te plaît. Celle de la vitre. La boulangère glisse la brioche dans un sac. Le papier craque, un peu gras. Merci. Merci. Raphaël tient le sac à deux mains. Le fond du sac est tiède. Elle est chaude, maman. Oui. Un grain de sucre sur ton pouce. Il brille. Tu le goûtes ? Il est sucré. Ils restent un moment près de la vitre. Raphaël dessine un petit rond du doigt. La brioche n'est plus floue, dehors. Elle est dans le sac, maintenant. On garde le sac au chaud. Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël avance trop vite vers le comptoir. La brioche, maintenant ! Sa voix se mélange à la cloche. Oh. Le torchon ne bouge pas. Le sourire ne revient pas. Raphaël refuse de foncer. Il recule d'un pas, près du bois. Tu veux venir près du bois ? Papa reste à sa hauteur. Raphaël écoute la cloche, un instant. Par la vitre, l'éclat de réverbère brille. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Une brioche, s'il te plaît. Celle de la vitre. Derrière le bois, une main se tend. Le papier enveloppe la brioche. Le sachet est chaud contre le manteau. Merci. Merci, Raphaël. Papa a entendu toute la phrase. Le ventre de Raphaël se desserre. Elle est chaude, maman. Tu as les mains dessus ? Oui, maman. Le papier est un peu gras, un peu tiède. Ça sent le beurre. On sort ? Oui, maman. Raphaël tient le sachet à deux mains. Le fond du sac est tiède.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Pascal a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;, s'il te plaît, merci. [pause]</t>
+          <t>Raphaël avance trop vite vers le comptoir. La brioche, maintenant ! Sa voix se mélange à la cloche. Oh. Le torchon ne bouge pas. Le sourire ne revient pas. Raphaël refuse de foncer. Il recule d'un pas, près du bois. Tu veux venir près du bois ? Papa reste à sa hauteur. Raphaël écoute la cloche, un instant. Par la vitre, l'éclat de réverbère brille. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Une brioche, s'il te plaît. Celle de la vitre. Derrière le bois, une main se tend. Le papier enveloppe la brioche. Le sachet est chaud contre le manteau. Merci. Merci, Raphaël. Papa a entendu toute la phrase. Le ventre de Raphaël se desserre. Elle est chaude, maman. Tu as les mains dessus ? Oui, maman. Le papier est un peu gras, un peu tiède. Ça sent le beurre. On sort ? Oui, maman. Raphaël tient le sachet à deux mains. Le fond du sac est tiède. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1629,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1637,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1663,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1695,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1711,38 +1743,48 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_salue_puis_demande; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
+          <t>narrateur|Raphaël avance trop vite vers le comptoir.
+enfant-m|La brioche, maintenant !
+narrateur|Sa voix se mélange à la cloche.
+enfant-m|Oh.
+narrateur|Le torchon ne bouge pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il recule d'un pas, près du bois.
+papa|Tu veux venir près du bois ?
+narrateur|Papa reste à sa hauteur.
+narrateur|Raphaël écoute la cloche, un instant.
+narrateur|Par la vitre, l'éclat de réverbère brille.
+enfant-m|Bonjour.
 maman|Bonjour.
 enfant-m|Une brioche, s'il te plaît.
 enfant-m|Celle de la vitre.
-narrateur|La boulangère glisse la brioche dans un sac.
-narrateur|Le papier craque, un peu gras.
+narrateur|Derrière le bois, une main se tend.
+narrateur|Le papier enveloppe la brioche.
+narrateur|Le sachet est chaud contre le manteau.
 enfant-m|Merci.
-papa|Merci.
-narrateur|Raphaël tient le sac à deux mains.
-narrateur|Le fond du sac est tiède.
+papa|Merci, Raphaël.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Raphaël se desserre.
 enfant-m|Elle est chaude, maman.
-maman|Oui.
-papa|Un grain de sucre sur ton pouce.
-enfant-m|Il brille.
-maman|Tu le goûtes ?
-enfant-m|Il est sucré.
-narrateur|Ils restent un moment près de la vitre.
-narrateur|Raphaël dessine un petit rond du doigt.
-narrateur|La brioche n'est plus floue, dehors.
-papa|Elle est dans le sac, maintenant.
-maman|On garde le sac au chaud.
-enfant-m|Oui, maman.</t>
+maman|Tu as les mains dessus ?
+enfant-m|Oui, maman.
+narrateur|Le papier est un peu gras, un peu tiède.
+enfant-m|Ça sent le beurre.
+maman|On sort ?
+enfant-m|Oui, maman.
+narrateur|Raphaël tient le sachet à deux mains.
+narrateur|Le fond du sac est tiède.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>papier</t>
+          <t>papier,cloche</t>
         </is>
       </c>
     </row>
@@ -1769,17 +1811,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent le long de la gouttière. Le seau est presque plein. Le parapluie goutte encore un peu. À la maison, maman ouvre le sac. La brioche sent le beurre, tout fort. Tu veux un bout ? Oui, papa. S'il te plaît. Raphaël croque. C'est doux. C'est un peu sucré. Merci, papa. Merci, Raphaël. Le sac vide reste sur la table, encore tiède. La gouttière chante moins, dehors. Le seau est plein. Oui. Et la brioche est à toi. Plus floue du tout.</t>
+          <t>Ils passent le pas de bois. La cloche fait ding. L'air mouillé revient sur les joues. Le vent de la rue prend le sachet. Le papier se gonfle, comme des ailes. Oh. Le sac près de la grille danse, lui aussi. Il s'envole, papa ! Les deux voix se mélangent. Le sac, Raphaël ? Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il ramène le sachet contre sa poitrine. Il écoute la rue, un instant. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On marche ? Oui, maman. Une goutte tombe du réverbère. Elle fait un rond dans la flaque. Comme le cercle jaune. Tu le vois, dans l'eau ? Oui, maman. Raphaël serre le sachet contre lui. Elle reste chaude. On rentre. Les pavés sont froids, un peu ronds. Je les entends, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent le long de la gouttière. Le seau est presque plein. Le parapluie goutte encore un peu. À la maison, maman ouvre le sac. La brioche sent le beurre, tout fort. Tu veux un bout ? Oui, papa. S'il te plaît. Raphaël croque. C'est doux. C'est un peu sucré. Merci, papa. Merci, Raphaël. Le sac vide reste sur la table, encore tiède. La gouttière chante moins, dehors. Le seau est plein. Oui. Et la brioche est à toi. Plus floue du tout.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils passent le pas de bois. La cloche fait ding. L'air mouillé revient sur les joues. Le vent de la rue prend le &lt;emphasis level="moderate"&gt;sachet&lt;/emphasis&gt;. Le papier se gonfle, comme des ailes. Oh. Le sac près de la grille danse, lui aussi. Il s'envole, papa ! Les deux voix se mélangent. Le sac, Raphaël ? Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il ramène le sachet contre sa poitrine. Il écoute la rue, un instant. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On marche ? Oui, maman. Une goutte tombe du réverbère. Elle fait un rond dans la flaque. Comme le cercle jaune. Tu le vois, dans l'eau ? Oui, maman. Raphaël serre le sachet contre lui. Elle reste chaude. On rentre. Les pavés sont froids, un peu ronds. Je les entends, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman ouvre le sac. Pascal sent la brioche. [pause]</t>
+          <t>Ils passent le pas de bois. La cloche fait ding. L'air mouillé revient sur les joues. Le vent de la rue prend le &lt;emphasis&gt;sachet&lt;/emphasis&gt;. Le papier se gonfle, comme des ailes. Oh. Le sac près de la grille danse, lui aussi. Il s'envole, papa ! Les deux voix se mélangent. Le sac, Raphaël ? Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il ramène le sachet contre sa poitrine. Il écoute la rue, un instant. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On marche ? Oui, maman. Une goutte tombe du réverbère. Elle fait un rond dans la flaque. Comme le cercle jaune. Tu le vois, dans l'eau ? Oui, maman. Raphaël serre le sachet contre lui. Elle reste chaude. On rentre. Les pavés sont froids, un peu ronds. Je les entends, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1826,7 +1868,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1834,10 +1876,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1858,28 +1900,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>sachet</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,10 +1934,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,33 +1948,47 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_quand_le_vent_prend_le_sachet; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils rentrent le long de la gouttière.
-narrateur|Le seau est presque plein.
-narrateur|Le parapluie goutte encore un peu.
-narrateur|À la maison, maman ouvre le sac.
-narrateur|La brioche sent le beurre, tout fort.
-papa|Tu veux un bout ?
+          <t>narrateur|Ils passent le pas de bois.
+narrateur|La cloche fait ding.
+narrateur|L'air mouillé revient sur les joues.
+narrateur|Le vent de la rue prend le sachet.
+narrateur|Le papier se gonfle, comme des ailes.
+enfant-m|Oh.
+narrateur|Le sac près de la grille danse, lui aussi.
+enfant-m|Il s'envole, papa !
+narrateur|Les deux voix se mélangent.
+papa|Le sac, Raphaël ?
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il ramène le sachet contre sa poitrine.
+narrateur|Il écoute la rue, un instant.
+enfant-m|Il est chaud, papa.
+papa|Tu le portes jusqu'à la rue ?
 enfant-m|Oui, papa.
-enfant-m|S'il te plaît.
-narrateur|Raphaël croque.
-narrateur|C'est doux.
-narrateur|C'est un peu sucré.
-enfant-m|Merci, papa.
-maman|Merci, Raphaël.
-narrateur|Le sac vide reste sur la table, encore tiède.
-papa|La gouttière chante moins, dehors.
-enfant-m|Le seau est plein.
-maman|Oui.
-maman|Et la brioche est à toi.
-papa|Plus floue du tout.</t>
+maman|On marche ?
+enfant-m|Oui, maman.
+narrateur|Une goutte tombe du réverbère.
+narrateur|Elle fait un rond dans la flaque.
+enfant-m|Comme le cercle jaune.
+maman|Tu le vois, dans l'eau ?
+enfant-m|Oui, maman.
+narrateur|Raphaël serre le sachet contre lui.
+enfant-m|Elle reste chaude.
+papa|On rentre.
+narrateur|Les pavés sont froids, un peu ronds.
+enfant-m|Je les entends, papa.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>pas,papier</t>
         </is>
       </c>
     </row>
@@ -1955,17 +2015,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sac tiède repose sur la table. Il reste un bout, un peu sucré. Bonne soirée, Raphaël. Elle n'est plus floue, ta brioche.</t>
+          <t>Ils s'arrêtent sous le réverbère jaune. La flaque tient son cercle, dans l'eau. Le sac de la grille ne danse plus. Le tien est fermé. Oui, papa. On est bien, ici. Ça sent le beurre, maman. Il est contre toi. Une vapeur monte du papier. Raphaël respire, plus large. On rentre ? Oui. Les joues de Raphaël se réchauffent. Le sachet reste tiède sous la main. L'éclat de réverbère tient sur le verre.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sac tiède repose sur la table. Il reste un bout, un peu sucré. Bonne soirée, Raphaël. Elle n'est plus floue, ta brioche.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent sous le réverbère jaune. La flaque tient son cercle, dans l'eau. Le sac de la grille ne danse plus. Le tien est fermé. Oui, papa. On est bien, ici. Ça sent le beurre, maman. Il est contre toi. Une vapeur monte du papier. Raphaël respire, plus large. On rentre ? Oui. Les joues de Raphaël se réchauffent. Le sachet reste tiède sous la main. L'&lt;emphasis level="moderate"&gt;éclat de réverbère&lt;/emphasis&gt; tient sur le verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent sous le réverbère jaune. La flaque tient son cercle, dans l'eau. Le sac de la grille ne danse plus. Le tien est fermé. Oui, papa. On est bien, ici. Ça sent le beurre, maman. Il est contre toi. Une vapeur monte du papier. Raphaël respire, plus large. On rentre ? Oui. Les joues de Raphaël se réchauffent. Le sachet reste tiède sous la main. L'&lt;emphasis&gt;éclat de réverbère&lt;/emphasis&gt; tient sur le verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2012,7 +2072,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2020,10 +2080,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2032,12 +2092,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2046,17 +2106,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de réverbère</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2065,11 +2129,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2078,27 +2142,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_verre; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sac tiède repose sur la table.
-narrateur|Il reste un bout, un peu sucré.
-maman|Bonne soirée, Raphaël.
-papa|Elle n'est plus floue, ta brioche.</t>
+          <t>narrateur|Ils s'arrêtent sous le réverbère jaune.
+narrateur|La flaque tient son cercle, dans l'eau.
+enfant-m|Le sac de la grille ne danse plus.
+papa|Le tien est fermé.
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+enfant-m|Ça sent le beurre, maman.
+maman|Il est contre toi.
+narrateur|Une vapeur monte du papier.
+narrateur|Raphaël respire, plus large.
+papa|On rentre ?
+enfant-m|Oui.
+narrateur|Les joues de Raphaël se réchauffent.
+narrateur|Le sachet reste tiède sous la main.
+narrateur|L'éclat de réverbère tient sur le verre.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pas</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2211,6 +2295,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>